<commit_message>
test script for login page
</commit_message>
<xml_diff>
--- a/Data/Akshara.xlsx
+++ b/Data/Akshara.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29910"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8FB9C069-D7BE-406E-9CA9-5BFDB883FE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50E38C75-F2E2-4983-BD27-3DEEB4EB8C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="valid_login" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -31,7 +32,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>student</t>
+  </si>
+  <si>
+    <t>Password123</t>
+  </si>
   <si>
     <t>Akshara</t>
   </si>
@@ -384,6 +397,36 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920A5A80-110E-42B4-9032-3CB87229A17C}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -393,7 +436,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>